<commit_message>
Guide people through the spreadsheets: blank sheets, a Start here tab, examples apart
Both downloads used to open with example numbers already filled in, so a
reader could take them for their own.

- Net Worth Calculator and Money Map spreadsheets now open on a "Start
  here" tab: what it does, step-by-step use, where to find each number
  (bank and PFA apps, loan balances, ajo organiser), phone tips, privacy.
- The user's own sheet ("My net worth" / "My Money Map") starts empty;
  the filled-in numbers moved to a clearly marked "Example" tab.
- The quarterly history no longer copies today's totals by formula: you
  type each quarter in, so past quarters stay put.
- Each download page shows "How to use it" steps and a privacy note; the
  net worth study explains the steps; the preview image shows the example.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kkM6oN9Y7js9B3i7hPKTM
</commit_message>
<xml_diff>
--- a/public/magnets/net-worth-calculator.xlsx
+++ b/public/magnets/net-worth-calculator.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Net worth" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly history" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="My net worth" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly history" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;₦&quot;#,##0;[Red]-&quot;₦&quot;#,##0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,19 +36,32 @@
       <sz val="18"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="0010302A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="004C6A62"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00D9822B"/>
+    </font>
+    <font>
       <i val="1"/>
+      <color rgb="004C6A62"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
       <color rgb="004C6A62"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <color rgb="004C6A62"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -58,19 +73,22 @@
       <sz val="13"/>
     </font>
     <font>
-      <i val="1"/>
-    </font>
-    <font>
-      <color rgb="004C6A62"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00D9822B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00D9822B"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -79,17 +97,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0010302A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4CC"/>
+        <fgColor rgb="00EEF2EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2EA"/>
+        <fgColor rgb="00D9822B"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,26 +128,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,417 +644,583 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="B1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Net Worth Calculator: start here</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>What this does</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Your net worth is what you own minus what you owe. It is the most honest number in personal finance: it shows what you have actually built, which a salary never does. This sheet adds it up for you and keeps a record every quarter so you can see whether it is rising.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>How to use it (about 20 minutes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1. Open the "My net worth" tab (at the bottom of the screen on a phone). It starts empty: these are YOUR numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2. Type today's date at the top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>3. Step 1, what you own: type a number in each yellow cell that applies to you. Leave the rest empty. Use today's value: what you would get if you sold or cashed it in today, not what you paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>4. In the "Pays you?" column, choose Yes for things that earn you money (savings with interest, pension, investments, tools you work with) and No for things that cost you money.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>5. Step 2, what you owe: type the balance LEFT to pay on every debt, not the original amount. Include loan apps, instalments, salary advances and money owed to family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>6. Step 3 shows your net worth straight away. If it is negative, that is common and fine. It is your starting point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>7. Open the "Quarterly history" tab and type your total assets and total liabilities in the row for this quarter. The change and the chart work themselves out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>8. Every 3 months (end of March, June, September, December), update "My net worth" and add a new row to the history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Where to find your numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Bank and mobile money balances: your banking apps. Pension: your Pension Fund Administrator (PFA) app, website or statement. Loans: your bank or loan app shows the amount outstanding. Ajo, esusu or cooperative: ask the organiser what you would collect. If you are not sure of a value, a careful estimate is fine. Write it down and correct it next time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Only type in the yellow cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>The white cells with totals hold formulas that do the maths. If you type over one by mistake, download a fresh copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Want to see a finished one first?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Open the "Example" tab. It shows Mercy's numbers filled in. Don't type your own numbers there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>On a phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Open the file with the free Google Sheets or Microsoft Excel app. In Google Sheets, tap File &gt; Make a copy (or Save as Google Sheets) so you can edit it and keep it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Your privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>This file stays on your phone or computer. Nobody else sees your numbers, and you never need to send them to anyone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>From the free Financial Intelligence class: kopkad.ng/blog. For educational purposes only. This is not financial advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>With Snowball, we keep it rolling.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0010302A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your Net Worth</t>
+          <t>My net worth</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>What you own − what you owe. Replace the example numbers in the yellow cells with yours, at today's value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>1. What you own (assets)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Type your own numbers in the yellow cells only. Everything else works itself out. New here? Read the "Start here" tab first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Write today's date, so you can compare next time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Step 1. What you own (assets)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Pays you?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cash in bank and mobile money</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>70000</v>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Where to find this number</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Savings plans, ajo or cooperative savings</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>350000</v>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>What you will get back</t>
+          <t>Cash in bank and mobile money</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Your balances today, from your bank and mobile money apps</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pension (Retirement Savings Account)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>380000</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>From your PFA statement or app</t>
+          <t>Savings plans, ajo or cooperative savings</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>What you would get back if you collected it today</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Investments (T-bills, fixed deposits, shares, funds)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr"/>
+          <t>Pension (Retirement Savings Account)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Your PFA app, website or latest statement</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Land or property</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Use the price you paid, not a hopeful value</t>
+          <t>Investments (T-bills, fixed deposits, shares, funds)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Current value from your bank or investment app</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Business stock and equipment</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Only if you use it to earn</t>
+          <t>Land or property</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>The price you paid, not a hopeful value</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Car or motorbike</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>What it would sell for today. "Yes" only if it earns for you</t>
+          <t>Business stock and equipment</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>What you could sell it for today. "Yes" only if you use it to earn</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Phone, laptop and other valuables</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>150000</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>What they would sell for today</t>
+          <t>Car or motorbike</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>What it would sell for today. "Yes" only if it earns money for you</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Phone, laptop and other valuables</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>What they would sell for today, not what you paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Money owed to you</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Only what you really expect to get back</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Total assets</t>
-        </is>
-      </c>
-      <c r="B14" s="8">
-        <f>SUM(B5:B13)</f>
-        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>Total assets</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
+        <f>SUM(B6:B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>Assets that pay you</t>
         </is>
       </c>
-      <c r="B15" s="8">
-        <f>SUMIF(C5:C13,"Yes",B5:B13)</f>
-        <v/>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Savings, pension, investments, tools you earn with: the part of your wealth that works for you</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>2. What you owe (liabilities)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B16" s="13">
+        <f>SUMIF(C6:C14,"Yes",B6:B14)</f>
+        <v/>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>The part of your wealth that works for you: savings, pension, investments, tools you earn with</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Step 2. What you owe (liabilities)</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Bank loans</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Balance left, not the original amount</t>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Where to find this number</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Loan apps</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="6" t="inlineStr"/>
+          <t>Bank loans</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>The balance left to pay, not the original loan. Check your bank app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Buy now, pay later / instalments</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Phones, appliances, furniture</t>
+          <t>Loan apps</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n"/>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>The amount the app says you owe today, including fees</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Salary advances</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr"/>
+          <t>Buy now, pay later / instalments</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Phones, appliances, furniture: what is left to pay</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Credit from traders or suppliers</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="6" t="inlineStr"/>
+          <t>Salary advances</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n"/>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>From your payslip or HR</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Money owed to family or friends</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Count it, even with no interest</t>
+          <t>Credit from traders or suppliers</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n"/>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Goods taken on credit and not yet paid for</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Unpaid bills (school fees, rent arrears, utilities)</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="6" t="inlineStr"/>
+          <t>Money owed to family or friends</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n"/>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Count it, even if there is no interest</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Unpaid bills (school fees, rent arrears, utilities)</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n"/>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Anything overdue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Other debts</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="B26" s="11" t="n"/>
+      <c r="D26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B26" s="8">
-        <f>SUM(B18:B25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>3. Your net worth</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="B27" s="13">
+        <f>SUM(B19:B26)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Step 3. Your net worth</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Net worth (assets − liabilities)</t>
         </is>
       </c>
-      <c r="B29" s="10">
-        <f>B14-B26</f>
-        <v/>
-      </c>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Negative is common, and it is a starting point, not a verdict. Watch the direction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>Next: copy your totals into the "Quarterly history" tab every 3 months (end of March, June, September, December).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="B30" s="15">
+        <f>B15-B27</f>
+        <v/>
+      </c>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Red and negative is common. It is a starting point, not a verdict. Watch the direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Step 4. Copy your totals into the "Quarterly history" tab, and do this again every 3 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Free from the Financial Intelligence class · kopkad.ng/blog</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>For educational purposes only. This is not financial advice.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>With Snowball, we keep it rolling.</t>
         </is>
@@ -1024,7 +1228,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1032,7 +1236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1051,39 +1255,39 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your net worth, every quarter</t>
+          <t>Quarterly history</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Twenty minutes, four times a year. Type your totals in the yellow cells; the rest works itself out.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Every 3 months, type your total assets and total liabilities from the "My net worth" tab into the yellow cells for that quarter.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Net worth</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
@@ -1095,19 +1299,13 @@
           <t>Dec 2026</t>
         </is>
       </c>
-      <c r="B5" s="4">
-        <f>'Net worth'!B14</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>'Net worth'!B26</f>
-        <v/>
-      </c>
-      <c r="D5" s="8">
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="13">
         <f>IF(AND(B5="",C5=""),"",B5-C5)</f>
         <v/>
       </c>
-      <c r="E5" s="16" t="inlineStr"/>
+      <c r="E5" s="20" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1115,13 +1313,13 @@
           <t>Mar 2027</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="8">
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="13">
         <f>IF(AND(B6="",C6=""),"",B6-C6)</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="20">
         <f>IF(OR(D6="",D5=""),"",D6-D5)</f>
         <v/>
       </c>
@@ -1132,13 +1330,13 @@
           <t>Jun 2027</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="8">
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="13">
         <f>IF(AND(B7="",C7=""),"",B7-C7)</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="20">
         <f>IF(OR(D7="",D6=""),"",D7-D6)</f>
         <v/>
       </c>
@@ -1149,13 +1347,13 @@
           <t>Sep 2027</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="8">
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="13">
         <f>IF(AND(B8="",C8=""),"",B8-C8)</f>
         <v/>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="20">
         <f>IF(OR(D8="",D7=""),"",D8-D7)</f>
         <v/>
       </c>
@@ -1166,13 +1364,13 @@
           <t>Dec 2027</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="8">
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="13">
         <f>IF(AND(B9="",C9=""),"",B9-C9)</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="20">
         <f>IF(OR(D9="",D8=""),"",D9-D8)</f>
         <v/>
       </c>
@@ -1183,13 +1381,13 @@
           <t>Mar 2028</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="8">
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="13">
         <f>IF(AND(B10="",C10=""),"",B10-C10)</f>
         <v/>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="20">
         <f>IF(OR(D10="",D9=""),"",D10-D9)</f>
         <v/>
       </c>
@@ -1200,13 +1398,13 @@
           <t>Jun 2028</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="8">
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="13">
         <f>IF(AND(B11="",C11=""),"",B11-C11)</f>
         <v/>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="20">
         <f>IF(OR(D11="",D10=""),"",D11-D10)</f>
         <v/>
       </c>
@@ -1217,13 +1415,13 @@
           <t>Sep 2028</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="8">
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="13">
         <f>IF(AND(B12="",C12=""),"",B12-C12)</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="20">
         <f>IF(OR(D12="",D11=""),"",D12-D11)</f>
         <v/>
       </c>
@@ -1234,21 +1432,21 @@
           <t>Dec 2028</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="8">
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="13">
         <f>IF(AND(B13="",C13=""),"",B13-C13)</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="20">
         <f>IF(OR(D13="",D12=""),"",D13-D12)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>The first row reads today's totals from the "Net worth" tab. From next quarter, type the new totals in.</t>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Started in a different month? Type over the quarter names in column A.</t>
         </is>
       </c>
     </row>
@@ -1256,4 +1454,481 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00D9822B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Mercy's net worth</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="n"/>
+      <c r="C1" s="22" t="n"/>
+      <c r="D1" s="22" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>This is an example to show you what a finished sheet looks like. Fill in your own on the "My net worth" tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>11 Dec 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Write today's date, so you can compare next time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Step 1. What you own (assets)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Pays you?</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Where to find this number</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cash in bank and mobile money</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>70000</v>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Your balances today, from your bank and mobile money apps</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Savings plans, ajo or cooperative savings</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>What you would get back if you collected it today</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pension (Retirement Savings Account)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>380000</v>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Your PFA app, website or latest statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Investments (T-bills, fixed deposits, shares, funds)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Current value from your bank or investment app</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Land or property</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>The price you paid, not a hopeful value</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Business stock and equipment</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>What you could sell it for today. "Yes" only if you use it to earn</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Car or motorbike</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>What it would sell for today. "Yes" only if it earns money for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Phone, laptop and other valuables</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>What they would sell for today, not what you paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Money owed to you</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Only what you really expect to get back</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Total assets</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
+        <f>SUM(B6:B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Assets that pay you</t>
+        </is>
+      </c>
+      <c r="B16" s="13">
+        <f>SUMIF(C6:C14,"Yes",B6:B14)</f>
+        <v/>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>The part of your wealth that works for you: savings, pension, investments, tools you earn with</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Step 2. What you owe (liabilities)</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Where to find this number</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bank loans</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>The balance left to pay, not the original loan. Check your bank app</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Loan apps</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>The amount the app says you owe today, including fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Buy now, pay later / instalments</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Phones, appliances, furniture: what is left to pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Salary advances</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>From your payslip or HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Credit from traders or suppliers</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Goods taken on credit and not yet paid for</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Money owed to family or friends</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Count it, even if there is no interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Unpaid bills (school fees, rent arrears, utilities)</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Anything overdue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Other debts</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Total liabilities</t>
+        </is>
+      </c>
+      <c r="B27" s="13">
+        <f>SUM(B19:B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Step 3. Your net worth</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Net worth (assets − liabilities)</t>
+        </is>
+      </c>
+      <c r="B30" s="15">
+        <f>B15-B27</f>
+        <v/>
+      </c>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Red and negative is common. It is a starting point, not a verdict. Watch the direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Step 4. Copy your totals into the "Quarterly history" tab, and do this again every 3 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Free from the Financial Intelligence class · kopkad.ng/blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>For educational purposes only. This is not financial advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>With Snowball, we keep it rolling.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>